<commit_message>
tudo funcionando, docker ainda não testado
</commit_message>
<xml_diff>
--- a/app/constants/dataset demo.xlsx
+++ b/app/constants/dataset demo.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="accounts" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2880" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2879" uniqueCount="180">
   <si>
     <t xml:space="preserve">bank_id</t>
   </si>
@@ -37,9 +37,6 @@
   </si>
   <si>
     <t xml:space="preserve">start_value </t>
-  </si>
-  <si>
-    <t xml:space="preserve">account_id</t>
   </si>
   <si>
     <t xml:space="preserve">Nubank</t>
@@ -70,6 +67,9 @@
   </si>
   <si>
     <t xml:space="preserve">category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">account_id</t>
   </si>
   <si>
     <t xml:space="preserve">is_active</t>
@@ -816,7 +816,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.7"/>
@@ -835,24 +835,18 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="D2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -861,53 +855,44 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1" t="n">
         <f aca="false">_xlfn.ORG.LIBREOFFICE.RAND.NV()*10000</f>
         <v>9425.22774570755</v>
       </c>
-      <c r="E3" s="1" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" s="1" t="n">
         <f aca="false">_xlfn.ORG.LIBREOFFICE.RAND.NV()*10000</f>
         <v>1013.59490012521</v>
       </c>
-      <c r="E4" s="1" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="D5" s="1" t="n">
         <f aca="false">_xlfn.ORG.LIBREOFFICE.RAND.NV()*10000</f>
         <v>4997.14606092546</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -934,19 +919,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>15</v>
@@ -966,7 +951,7 @@
         <v>17</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>1</v>
@@ -986,7 +971,7 @@
         <v>17</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>1</v>
@@ -1006,7 +991,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>1</v>
@@ -1026,7 +1011,7 @@
         <v>21</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>1</v>
@@ -1046,7 +1031,7 @@
         <v>23</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>1</v>
@@ -1066,7 +1051,7 @@
         <v>21</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>1</v>
@@ -1100,19 +1085,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>26</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>27</v>

</xml_diff>